<commit_message>
feat(email): add white logo and table layout for proper rendering
</commit_message>
<xml_diff>
--- a/File di origine/Competizioni.xlsx
+++ b/File di origine/Competizioni.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\Downloads\Antigravity\Dance Manager\File di origine\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA1B0A15-BCA3-410B-89AD-3186E61CAB5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BF3AA88-420C-4438-A16A-97417B57CAA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{80788694-69B5-4A11-9D9B-990EA002F532}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Nome</t>
   </si>
@@ -54,40 +54,7 @@
     <t>descrizione</t>
   </si>
   <si>
-    <t>The Star Championship</t>
-  </si>
-  <si>
-    <t>Palaeventi Pieve di Cento</t>
-  </si>
-  <si>
-    <t>Competizione Internazionale</t>
-  </si>
-  <si>
-    <t>Syllabus di Copparo</t>
-  </si>
-  <si>
-    <t>Copparo</t>
-  </si>
-  <si>
     <t>data aumento quota</t>
-  </si>
-  <si>
-    <t>Syllabus Marche</t>
-  </si>
-  <si>
-    <t>Marche</t>
-  </si>
-  <si>
-    <t>Star Cup - Verona</t>
-  </si>
-  <si>
-    <t>Verona</t>
-  </si>
-  <si>
-    <t>FEINDA</t>
-  </si>
-  <si>
-    <t>Cervia</t>
   </si>
 </sst>
 </file>
@@ -484,126 +451,56 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="2">
-        <v>46092</v>
-      </c>
-      <c r="C2" s="2">
-        <v>46096</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="2">
-        <v>46063</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46082</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>8</v>
-      </c>
+      <c r="A2" s="1"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="1"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="2">
-        <v>46124</v>
-      </c>
-      <c r="C3" s="2">
-        <v>46124</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="2">
-        <v>46092</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46114</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>8</v>
-      </c>
+      <c r="A3" s="1"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="1"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="2">
-        <v>46068</v>
-      </c>
-      <c r="C4" s="2">
-        <v>46068</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="2">
-        <v>46065</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46066</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>8</v>
-      </c>
+      <c r="A4" s="1"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="1"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="2">
-        <v>46154</v>
-      </c>
-      <c r="C5" s="2">
-        <v>46155</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="2">
-        <v>46154</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46155</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>8</v>
-      </c>
+      <c r="A5" s="1"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="1"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="2">
-        <v>46174</v>
-      </c>
-      <c r="C6" s="2">
-        <v>46174</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E6" s="2">
-        <v>46143</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46143</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>8</v>
-      </c>
+      <c r="A6" s="1"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="1"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>

</xml_diff>